<commit_message>
Add homepage and all-captures Wayback links to the sample
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9K4kXodKmqW5FKv8B7Kmh
</commit_message>
<xml_diff>
--- a/research/fl-voucher/data/processed/wayback_sample30.xlsx
+++ b/research/fl-voucher/data/processed/wayback_sample30.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB31"/>
+  <dimension ref="A1:BI31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,187 +517,222 @@
           <t>wayback_2026_link</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_2021_home_link</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_2022_home_link</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_2023_home_link</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_2024_home_link</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_2025_home_link</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_2026_home_link</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>wayback_all_captures_link</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>2021_page_year_printed</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>2021_elem</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>2021_mid</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>2021_high</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>2021_overall</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>2021_snapshot_date</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>2022_page_year_printed</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>2022_elem</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>2022_mid</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>2022_high</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>2022_overall</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>2022_snapshot_date</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>2023_page_year_printed</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>2023_elem</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>2023_mid</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>2023_high</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>2023_overall</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>2023_snapshot_date</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>2024_page_year_printed</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AR1" s="2" t="inlineStr">
         <is>
           <t>2024_elem</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AS1" s="2" t="inlineStr">
         <is>
           <t>2024_mid</t>
         </is>
       </c>
-      <c r="AM1" s="2" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>2024_high</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>2024_overall</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="AV1" s="2" t="inlineStr">
         <is>
           <t>2024_snapshot_date</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>2025_page_year_printed</t>
         </is>
       </c>
-      <c r="AQ1" s="2" t="inlineStr">
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>2025_elem</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
         <is>
           <t>2025_mid</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="AZ1" s="2" t="inlineStr">
         <is>
           <t>2025_high</t>
         </is>
       </c>
-      <c r="AT1" s="2" t="inlineStr">
+      <c r="BA1" s="2" t="inlineStr">
         <is>
           <t>2025_overall</t>
         </is>
       </c>
-      <c r="AU1" s="2" t="inlineStr">
+      <c r="BB1" s="2" t="inlineStr">
         <is>
           <t>2025_snapshot_date</t>
         </is>
       </c>
-      <c r="AV1" s="2" t="inlineStr">
+      <c r="BC1" s="2" t="inlineStr">
         <is>
           <t>2026_page_year_printed</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>2026_elem</t>
         </is>
       </c>
-      <c r="AX1" s="2" t="inlineStr">
+      <c r="BE1" s="2" t="inlineStr">
         <is>
           <t>2026_mid</t>
         </is>
       </c>
-      <c r="AY1" s="2" t="inlineStr">
+      <c r="BF1" s="2" t="inlineStr">
         <is>
           <t>2026_high</t>
         </is>
       </c>
-      <c r="AZ1" s="2" t="inlineStr">
+      <c r="BG1" s="2" t="inlineStr">
         <is>
           <t>2026_overall</t>
         </is>
       </c>
-      <c r="BA1" s="2" t="inlineStr">
+      <c r="BH1" s="2" t="inlineStr">
         <is>
           <t>2026_snapshot_date</t>
         </is>
       </c>
-      <c r="BB1" s="2" t="inlineStr">
+      <c r="BI1" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -749,41 +784,69 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
@@ -814,6 +877,13 @@
       <c r="AZ2" t="inlineStr"/>
       <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -861,41 +931,69 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
@@ -926,6 +1024,13 @@
       <c r="AZ3" t="inlineStr"/>
       <c r="BA3" t="inlineStr"/>
       <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -973,41 +1078,69 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
@@ -1038,6 +1171,13 @@
       <c r="AZ4" t="inlineStr"/>
       <c r="BA4" t="inlineStr"/>
       <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1085,41 +1225,69 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X5" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
@@ -1150,6 +1318,13 @@
       <c r="AZ5" t="inlineStr"/>
       <c r="BA5" t="inlineStr"/>
       <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1197,41 +1372,69 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X6" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
@@ -1262,6 +1465,13 @@
       <c r="AZ6" t="inlineStr"/>
       <c r="BA6" t="inlineStr"/>
       <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1317,41 +1527,69 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
@@ -1382,6 +1620,13 @@
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1429,41 +1674,69 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S8" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr"/>
@@ -1494,6 +1767,13 @@
       <c r="AZ8" t="inlineStr"/>
       <c r="BA8" t="inlineStr"/>
       <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
+      <c r="BI8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1541,41 +1821,69 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U9" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W9" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X9" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr"/>
@@ -1606,6 +1914,13 @@
       <c r="AZ9" t="inlineStr"/>
       <c r="BA9" t="inlineStr"/>
       <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
+      <c r="BI9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1661,41 +1976,69 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U10" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W10" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X10" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>
@@ -1726,6 +2069,13 @@
       <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr"/>
+      <c r="BI10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1773,41 +2123,69 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S11" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V11" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W11" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X11" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
@@ -1838,6 +2216,13 @@
       <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="inlineStr"/>
       <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr"/>
+      <c r="BI11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1885,41 +2270,69 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W12" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X12" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
@@ -1950,6 +2363,13 @@
       <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="inlineStr"/>
       <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="inlineStr"/>
+      <c r="BH12" t="inlineStr"/>
+      <c r="BI12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1997,41 +2417,69 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V13" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W13" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X13" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr"/>
@@ -2062,6 +2510,13 @@
       <c r="AZ13" t="inlineStr"/>
       <c r="BA13" t="inlineStr"/>
       <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2113,41 +2568,69 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W14" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr"/>
@@ -2178,6 +2661,13 @@
       <c r="AZ14" t="inlineStr"/>
       <c r="BA14" t="inlineStr"/>
       <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr"/>
+      <c r="BH14" t="inlineStr"/>
+      <c r="BI14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2233,41 +2723,69 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W15" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X15" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
@@ -2298,6 +2816,13 @@
       <c r="AZ15" t="inlineStr"/>
       <c r="BA15" t="inlineStr"/>
       <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr"/>
+      <c r="BI15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2345,41 +2870,69 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V16" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W16" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X16" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr"/>
@@ -2410,6 +2963,13 @@
       <c r="AZ16" t="inlineStr"/>
       <c r="BA16" t="inlineStr"/>
       <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr"/>
+      <c r="BI16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2457,41 +3017,69 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V17" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W17" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X17" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr"/>
@@ -2522,6 +3110,13 @@
       <c r="AZ17" t="inlineStr"/>
       <c r="BA17" t="inlineStr"/>
       <c r="BB17" t="inlineStr"/>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr"/>
+      <c r="BH17" t="inlineStr"/>
+      <c r="BI17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2569,41 +3164,69 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V18" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W18" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X18" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr"/>
@@ -2634,6 +3257,13 @@
       <c r="AZ18" t="inlineStr"/>
       <c r="BA18" t="inlineStr"/>
       <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr"/>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2681,41 +3311,69 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V19" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W19" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X19" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
       <c r="AA19" t="inlineStr"/>
@@ -2746,6 +3404,13 @@
       <c r="AZ19" t="inlineStr"/>
       <c r="BA19" t="inlineStr"/>
       <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2797,41 +3462,69 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V20" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W20" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X20" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
       <c r="AA20" t="inlineStr"/>
@@ -2862,6 +3555,13 @@
       <c r="AZ20" t="inlineStr"/>
       <c r="BA20" t="inlineStr"/>
       <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
+      <c r="BG20" t="inlineStr"/>
+      <c r="BH20" t="inlineStr"/>
+      <c r="BI20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2917,41 +3617,69 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V21" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W21" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X21" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr"/>
@@ -2982,6 +3710,13 @@
       <c r="AZ21" t="inlineStr"/>
       <c r="BA21" t="inlineStr"/>
       <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3029,41 +3764,69 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V22" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W22" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X22" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
@@ -3094,6 +3857,13 @@
       <c r="AZ22" t="inlineStr"/>
       <c r="BA22" t="inlineStr"/>
       <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr"/>
+      <c r="BG22" t="inlineStr"/>
+      <c r="BH22" t="inlineStr"/>
+      <c r="BI22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3149,41 +3919,69 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V23" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W23" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X23" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr"/>
@@ -3214,6 +4012,13 @@
       <c r="AZ23" t="inlineStr"/>
       <c r="BA23" t="inlineStr"/>
       <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
+      <c r="BG23" t="inlineStr"/>
+      <c r="BH23" t="inlineStr"/>
+      <c r="BI23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3269,41 +4074,69 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U24" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V24" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W24" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X24" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
@@ -3334,6 +4167,13 @@
       <c r="AZ24" t="inlineStr"/>
       <c r="BA24" t="inlineStr"/>
       <c r="BB24" t="inlineStr"/>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
+      <c r="BG24" t="inlineStr"/>
+      <c r="BH24" t="inlineStr"/>
+      <c r="BI24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3381,41 +4221,69 @@
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T25" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U25" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V25" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W25" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X25" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
@@ -3446,6 +4314,13 @@
       <c r="AZ25" t="inlineStr"/>
       <c r="BA25" t="inlineStr"/>
       <c r="BB25" t="inlineStr"/>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
+      <c r="BG25" t="inlineStr"/>
+      <c r="BH25" t="inlineStr"/>
+      <c r="BI25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3501,41 +4376,69 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U26" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V26" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W26" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X26" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr"/>
@@ -3566,6 +4469,13 @@
       <c r="AZ26" t="inlineStr"/>
       <c r="BA26" t="inlineStr"/>
       <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="inlineStr"/>
+      <c r="BF26" t="inlineStr"/>
+      <c r="BG26" t="inlineStr"/>
+      <c r="BH26" t="inlineStr"/>
+      <c r="BI26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3613,41 +4523,69 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S27" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U27" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V27" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W27" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X27" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
       <c r="AA27" t="inlineStr"/>
@@ -3678,6 +4616,13 @@
       <c r="AZ27" t="inlineStr"/>
       <c r="BA27" t="inlineStr"/>
       <c r="BB27" t="inlineStr"/>
+      <c r="BC27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="inlineStr"/>
+      <c r="BF27" t="inlineStr"/>
+      <c r="BG27" t="inlineStr"/>
+      <c r="BH27" t="inlineStr"/>
+      <c r="BI27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3733,41 +4678,69 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U28" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V28" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W28" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X28" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr"/>
@@ -3798,6 +4771,13 @@
       <c r="AZ28" t="inlineStr"/>
       <c r="BA28" t="inlineStr"/>
       <c r="BB28" t="inlineStr"/>
+      <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="inlineStr"/>
+      <c r="BF28" t="inlineStr"/>
+      <c r="BG28" t="inlineStr"/>
+      <c r="BH28" t="inlineStr"/>
+      <c r="BI28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3845,41 +4825,69 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S29" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T29" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U29" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V29" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W29" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X29" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr"/>
@@ -3910,6 +4918,13 @@
       <c r="AZ29" t="inlineStr"/>
       <c r="BA29" t="inlineStr"/>
       <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
+      <c r="BG29" t="inlineStr"/>
+      <c r="BH29" t="inlineStr"/>
+      <c r="BI29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3965,41 +4980,69 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U30" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V30" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W30" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X30" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr"/>
@@ -4030,6 +5073,13 @@
       <c r="AZ30" t="inlineStr"/>
       <c r="BA30" t="inlineStr"/>
       <c r="BB30" t="inlineStr"/>
+      <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="inlineStr"/>
+      <c r="BF30" t="inlineStr"/>
+      <c r="BG30" t="inlineStr"/>
+      <c r="BH30" t="inlineStr"/>
+      <c r="BI30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4085,41 +5135,69 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2021 page</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2022 page</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2023 page</t>
         </is>
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2024 page</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025 page</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
+          <t>2026 page</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="inlineStr">
+        <is>
+          <t>2021 home</t>
+        </is>
+      </c>
+      <c r="S31" s="3" t="inlineStr">
+        <is>
+          <t>2022 home</t>
+        </is>
+      </c>
+      <c r="T31" s="3" t="inlineStr">
+        <is>
+          <t>2023 home</t>
+        </is>
+      </c>
+      <c r="U31" s="3" t="inlineStr">
+        <is>
+          <t>2024 home</t>
+        </is>
+      </c>
+      <c r="V31" s="3" t="inlineStr">
+        <is>
+          <t>2025 home</t>
+        </is>
+      </c>
+      <c r="W31" s="3" t="inlineStr">
+        <is>
+          <t>2026 home</t>
+        </is>
+      </c>
+      <c r="X31" s="3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr"/>
@@ -4150,6 +5228,13 @@
       <c r="AZ31" t="inlineStr"/>
       <c r="BA31" t="inlineStr"/>
       <c r="BB31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="inlineStr"/>
+      <c r="BF31" t="inlineStr"/>
+      <c r="BG31" t="inlineStr"/>
+      <c r="BH31" t="inlineStr"/>
+      <c r="BI31" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4159,180 +5244,390 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R2" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T2" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U2" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R3" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S3" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T3" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U3" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R4" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T4" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V4" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R5" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T5" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V5" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R6" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S6" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T6" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V6" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V7" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T8" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V8" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W8" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T11" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V11" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V12" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T13" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U13" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V13" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W13" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T14" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V14" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W14" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V15" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W15" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V16" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W16" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R17" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T17" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W17" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W18" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T19" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W19" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T20" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W20" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T21" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V21" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W21" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V22" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W22" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T23" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V23" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W23" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T24" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V24" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W24" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R25" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T25" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V25" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W25" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T26" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V26" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W26" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T27" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V27" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W27" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T28" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V28" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W28" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R29" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T29" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V29" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W29" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R30" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T30" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V30" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W30" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R31" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T31" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W31" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId390"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>